<commit_message>
Fix and expand ISTG-INT[I2C] specialization
Corrects typos and grammar errors from original contribution.
Adds standard ISTG reference sources to all test cases, expands
tool coverage to include i2c-tools (i2cdetect/i2cdump), Bus Pirate,
and HydraBus. Adds safe-probe guidance for i2cdetect -r, i2cdump
addressing-width warning for large EEPROMs, and EEPROM WP pin test.
Adds ISTG-INT[I2C]-INFO-003 (EEPROM/Memory Extraction) as a new
test case. Expands INPV-001 to cover clock stretching DoS, repeated
START abuse, NAK flooding, and general call address probing.
Regenerates checklist with INFO-003 entry.
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="25800" yWindow="0" windowWidth="25800" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="2" min="1" max="1"/>
@@ -1665,12 +1665,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ISTG-PHY-AUTHZ-001</t>
+          <t>ISTG-INT[I2C]-AUTHZ-001</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1680,41 +1680,41 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Bus Interaction with Unauthorized Devices</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ISTG-PHY-AUTHZ-002</t>
+          <t>ISTG-INT[I2C]-INFO-001</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Slave Enumeration</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-001</t>
+          <t>ISTG-INT[I2C]-INFO-002</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1724,19 +1724,19 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Communication Sniffing</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-002</t>
+          <t>ISTG-INT[I2C]-INFO-003</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1746,36 +1746,36 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>EEPROM/Memory Extraction</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-003</t>
+          <t>ISTG-INT[I2C]-INPV-001</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Insufficient Handling of Invalid Data</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CONF-001</t>
+          <t>ISTG-PHY-AUTHZ-001</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1785,19 +1785,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CONF-002</t>
+          <t>ISTG-PHY-AUTHZ-002</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1807,19 +1807,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ISTG-PHY-SCRT-001</t>
+          <t>ISTG-PHY-INFO-001</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1829,19 +1829,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CRYPT-001</t>
+          <t>ISTG-PHY-INFO-002</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1851,19 +1851,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ISTG-PHY-LOGIC-001</t>
+          <t>ISTG-PHY-INFO-003</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1873,19 +1873,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INPV-001</t>
+          <t>ISTG-PHY-CONF-001</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1895,19 +1895,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INPV-002</t>
+          <t>ISTG-PHY-CONF-002</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1917,129 +1917,129 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-AUTHZ-001</t>
+          <t>ISTG-PHY-SCRT-001</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-AUTHZ-002</t>
+          <t>ISTG-PHY-CRYPT-001</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-001</t>
+          <t>ISTG-PHY-LOGIC-001</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-002</t>
+          <t>ISTG-PHY-INPV-001</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-003</t>
+          <t>ISTG-PHY-INPV-002</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CONF-001</t>
+          <t>ISTG-WRLS-AUTHZ-001</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CONF-002</t>
+          <t>ISTG-WRLS-AUTHZ-002</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2071,19 +2071,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-SCRT-001</t>
+          <t>ISTG-WRLS-INFO-001</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2093,19 +2093,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CRYPT-001</t>
+          <t>ISTG-WRLS-INFO-002</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2115,19 +2115,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-LOGIC-001</t>
+          <t>ISTG-WRLS-INFO-003</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2137,19 +2137,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INPV-001</t>
+          <t>ISTG-WRLS-CONF-001</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2159,19 +2159,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INPV-002</t>
+          <t>ISTG-WRLS-CONF-002</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2181,129 +2181,129 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ISTG-UI-AUTHZ-001</t>
+          <t>ISTG-WRLS-SCRT-001</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ISTG-UI-AUTHZ-002</t>
+          <t>ISTG-WRLS-CRYPT-001</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-001</t>
+          <t>ISTG-WRLS-LOGIC-001</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-002</t>
+          <t>ISTG-WRLS-INPV-001</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-003</t>
+          <t>ISTG-WRLS-INPV-002</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ISTG-UI-CONF-001</t>
+          <t>ISTG-UI-AUTHZ-001</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2313,19 +2313,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ISTG-UI-CONF-002</t>
+          <t>ISTG-UI-AUTHZ-002</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2335,19 +2335,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ISTG-UI-SCRT-001</t>
+          <t>ISTG-UI-INFO-001</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2357,19 +2357,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ISTG-UI-CRYPT-001</t>
+          <t>ISTG-UI-INFO-002</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2379,19 +2379,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ISTG-UI-LOGIC-001</t>
+          <t>ISTG-UI-INFO-003</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2401,19 +2401,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ISTG-UI-INPV-001</t>
+          <t>ISTG-UI-CONF-001</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2423,32 +2423,142 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>ISTG-UI-CONF-002</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Configuration and Patch Management</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Presence of Unnecessary Software and Functionalities</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ISTG-UI-SCRT-001</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Secrets</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Access to Confidential Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ISTG-UI-CRYPT-001</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Cryptography</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Usage of Weak Cryptographic Algorithms</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ISTG-UI-LOGIC-001</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Business Logic</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Circumvention of the Intended Business Logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ISTG-UI-INPV-001</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Input Validation</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Insufficient Input Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>ISTG-UI-INPV-002</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>User Interfaces</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Input Validation</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>Code or Command Injection</t>
         </is>

</xml_diff>

<commit_message>
Add JTAG specialization to spreadsheet checklist
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="2" min="1" max="1"/>
@@ -1665,12 +1665,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ISTG-PHY-AUTHZ-001</t>
+          <t>ISTG-INT[JTAG]-AUTHZ-001</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Internal Interfaces</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1680,19 +1680,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Unauthorized Debug Access in Production State</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ISTG-PHY-AUTHZ-002</t>
+          <t>ISTG-INT[JTAG]-AUTHZ-002</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Internal Interfaces</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1702,19 +1702,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Early-Boot Debug-State Exposure</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-001</t>
+          <t>ISTG-INT[JTAG]-INFO-001</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Internal Interfaces</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1724,19 +1724,19 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Interface Presence, Physical Accessibility, and Transport Identification</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-002</t>
+          <t>ISTG-INT[JTAG]-INFO-002</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Internal Interfaces</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1746,36 +1746,36 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Accessible Asset Boundary Review</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-003</t>
+          <t>ISTG-INT[JTAG]-CONF-001</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Internal Interfaces</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Lifecycle and Security-Configuration Review</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CONF-001</t>
+          <t>ISTG-PHY-AUTHZ-001</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1785,19 +1785,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CONF-002</t>
+          <t>ISTG-PHY-AUTHZ-002</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1807,19 +1807,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ISTG-PHY-SCRT-001</t>
+          <t>ISTG-PHY-INFO-001</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1829,19 +1829,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CRYPT-001</t>
+          <t>ISTG-PHY-INFO-002</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1851,19 +1851,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ISTG-PHY-LOGIC-001</t>
+          <t>ISTG-PHY-INFO-003</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1873,19 +1873,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INPV-001</t>
+          <t>ISTG-PHY-CONF-001</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1895,19 +1895,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INPV-002</t>
+          <t>ISTG-PHY-CONF-002</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1917,129 +1917,129 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-AUTHZ-001</t>
+          <t>ISTG-PHY-SCRT-001</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-AUTHZ-002</t>
+          <t>ISTG-PHY-CRYPT-001</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-001</t>
+          <t>ISTG-PHY-LOGIC-001</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-002</t>
+          <t>ISTG-PHY-INPV-001</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-003</t>
+          <t>ISTG-PHY-INPV-002</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CONF-001</t>
+          <t>ISTG-WRLS-AUTHZ-001</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CONF-002</t>
+          <t>ISTG-WRLS-AUTHZ-002</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2071,19 +2071,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-SCRT-001</t>
+          <t>ISTG-WRLS-INFO-001</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2093,19 +2093,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CRYPT-001</t>
+          <t>ISTG-WRLS-INFO-002</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2115,19 +2115,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-LOGIC-001</t>
+          <t>ISTG-WRLS-INFO-003</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2137,19 +2137,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INPV-001</t>
+          <t>ISTG-WRLS-CONF-001</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2159,19 +2159,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INPV-002</t>
+          <t>ISTG-WRLS-CONF-002</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2181,129 +2181,129 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ISTG-UI-AUTHZ-001</t>
+          <t>ISTG-WRLS-SCRT-001</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ISTG-UI-AUTHZ-002</t>
+          <t>ISTG-WRLS-CRYPT-001</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-001</t>
+          <t>ISTG-WRLS-LOGIC-001</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-002</t>
+          <t>ISTG-WRLS-INPV-001</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-003</t>
+          <t>ISTG-WRLS-INPV-002</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ISTG-UI-CONF-001</t>
+          <t>ISTG-UI-AUTHZ-001</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2313,19 +2313,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ISTG-UI-CONF-002</t>
+          <t>ISTG-UI-AUTHZ-002</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2335,19 +2335,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ISTG-UI-SCRT-001</t>
+          <t>ISTG-UI-INFO-001</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2357,19 +2357,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ISTG-UI-CRYPT-001</t>
+          <t>ISTG-UI-INFO-002</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2379,19 +2379,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ISTG-UI-LOGIC-001</t>
+          <t>ISTG-UI-INFO-003</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2401,19 +2401,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ISTG-UI-INPV-001</t>
+          <t>ISTG-UI-CONF-001</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2423,32 +2423,142 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>ISTG-UI-CONF-002</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Configuration and Patch Management</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Presence of Unnecessary Software and Functionalities</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ISTG-UI-SCRT-001</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Secrets</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Access to Confidential Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ISTG-UI-CRYPT-001</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Cryptography</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Usage of Weak Cryptographic Algorithms</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ISTG-UI-LOGIC-001</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Business Logic</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Circumvention of the Intended Business Logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ISTG-UI-INPV-001</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Input Validation</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Insufficient Input Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>ISTG-UI-INPV-002</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>User Interfaces</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Input Validation</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>Code or Command Injection</t>
         </is>

</xml_diff>

<commit_message>
Add ISTG-INT[I2C] Inter-Integrated Circuit specialization (#24)
* Add new component specialization ISTG-INT[I2C]

* Fix and expand ISTG-INT[I2C] specialization

Corrects typos and grammar errors from original contribution.
Adds standard ISTG reference sources to all test cases, expands
tool coverage to include i2c-tools (i2cdetect/i2cdump), Bus Pirate,
and HydraBus. Adds safe-probe guidance for i2cdetect -r, i2cdump
addressing-width warning for large EEPROMs, and EEPROM WP pin test.
Adds ISTG-INT[I2C]-INFO-003 (EEPROM/Memory Extraction) as a new
test case. Expands INPV-001 to cover clock stretching DoS, repeated
START abuse, NAK flooding, and general call address probing.
Regenerates checklist with INFO-003 entry.

---------

Co-authored-by: nitrescov <nitrescov@protonmail.com>
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="25800" yWindow="0" windowWidth="25800" windowHeight="21000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F90"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="2" min="1" max="1"/>
@@ -1665,12 +1665,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ISTG-PHY-AUTHZ-001</t>
+          <t>ISTG-INT[I2C]-AUTHZ-001</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1680,41 +1680,41 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Bus Interaction with Unauthorized Devices</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ISTG-PHY-AUTHZ-002</t>
+          <t>ISTG-INT[I2C]-INFO-001</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Slave Enumeration</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-001</t>
+          <t>ISTG-INT[I2C]-INFO-002</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1724,19 +1724,19 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Communication Sniffing</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-002</t>
+          <t>ISTG-INT[I2C]-INFO-003</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1746,36 +1746,36 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>EEPROM/Memory Extraction</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-003</t>
+          <t>ISTG-INT[I2C]-INPV-001</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Insufficient Handling of Invalid Data</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CONF-001</t>
+          <t>ISTG-PHY-AUTHZ-001</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1785,19 +1785,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CONF-002</t>
+          <t>ISTG-PHY-AUTHZ-002</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1807,19 +1807,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ISTG-PHY-SCRT-001</t>
+          <t>ISTG-PHY-INFO-001</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1829,19 +1829,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CRYPT-001</t>
+          <t>ISTG-PHY-INFO-002</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1851,19 +1851,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ISTG-PHY-LOGIC-001</t>
+          <t>ISTG-PHY-INFO-003</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1873,19 +1873,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INPV-001</t>
+          <t>ISTG-PHY-CONF-001</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1895,19 +1895,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INPV-002</t>
+          <t>ISTG-PHY-CONF-002</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1917,129 +1917,129 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-AUTHZ-001</t>
+          <t>ISTG-PHY-SCRT-001</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-AUTHZ-002</t>
+          <t>ISTG-PHY-CRYPT-001</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-001</t>
+          <t>ISTG-PHY-LOGIC-001</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-002</t>
+          <t>ISTG-PHY-INPV-001</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-003</t>
+          <t>ISTG-PHY-INPV-002</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CONF-001</t>
+          <t>ISTG-WRLS-AUTHZ-001</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2049,19 +2049,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CONF-002</t>
+          <t>ISTG-WRLS-AUTHZ-002</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2071,19 +2071,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-SCRT-001</t>
+          <t>ISTG-WRLS-INFO-001</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2093,19 +2093,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CRYPT-001</t>
+          <t>ISTG-WRLS-INFO-002</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2115,19 +2115,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-LOGIC-001</t>
+          <t>ISTG-WRLS-INFO-003</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2137,19 +2137,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INPV-001</t>
+          <t>ISTG-WRLS-CONF-001</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2159,19 +2159,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INPV-002</t>
+          <t>ISTG-WRLS-CONF-002</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2181,129 +2181,129 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ISTG-UI-AUTHZ-001</t>
+          <t>ISTG-WRLS-SCRT-001</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ISTG-UI-AUTHZ-002</t>
+          <t>ISTG-WRLS-CRYPT-001</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-001</t>
+          <t>ISTG-WRLS-LOGIC-001</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-002</t>
+          <t>ISTG-WRLS-INPV-001</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-003</t>
+          <t>ISTG-WRLS-INPV-002</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ISTG-UI-CONF-001</t>
+          <t>ISTG-UI-AUTHZ-001</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2313,19 +2313,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ISTG-UI-CONF-002</t>
+          <t>ISTG-UI-AUTHZ-002</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2335,19 +2335,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ISTG-UI-SCRT-001</t>
+          <t>ISTG-UI-INFO-001</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2357,19 +2357,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ISTG-UI-CRYPT-001</t>
+          <t>ISTG-UI-INFO-002</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2379,19 +2379,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ISTG-UI-LOGIC-001</t>
+          <t>ISTG-UI-INFO-003</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2401,19 +2401,19 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ISTG-UI-INPV-001</t>
+          <t>ISTG-UI-CONF-001</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2423,32 +2423,142 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>ISTG-UI-CONF-002</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Configuration and Patch Management</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Presence of Unnecessary Software and Functionalities</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ISTG-UI-SCRT-001</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Secrets</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Access to Confidential Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ISTG-UI-CRYPT-001</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Cryptography</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Usage of Weak Cryptographic Algorithms</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ISTG-UI-LOGIC-001</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Business Logic</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Circumvention of the Intended Business Logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ISTG-UI-INPV-001</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Input Validation</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Insufficient Input Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>ISTG-UI-INPV-002</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>User Interfaces</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Input Validation</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>Code or Command Injection</t>
         </is>

</xml_diff>

<commit_message>
Prepare JTAG specialization for merge readiness
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" style="2" min="1" max="1"/>
@@ -675,7 +675,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ISTG-MEM-SCRT-001</t>
+          <t>ISTG-MEM-INFO-005</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -685,19 +685,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Unencrypted Storage of Secrets</t>
+          <t>Insecure Binary Compilation Options</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ISTG-MEM-CRYPT-001</t>
+          <t>ISTG-MEM-SCRT-001</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -707,41 +707,41 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Unencrypted Storage of Secrets</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ISTG-FW-INFO-001</t>
+          <t>ISTG-MEM-CRYPT-001</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>Memory</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Disclosure of Source Code and Binaries</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ISTG-FW-INFO-002</t>
+          <t>ISTG-FW-INFO-001</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -756,14 +756,14 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Disclosure of Source Code and Binaries</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ISTG-FW-INFO-003</t>
+          <t>ISTG-FW-INFO-002</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -778,14 +778,14 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ISTG-FW-CONF-001</t>
+          <t>ISTG-FW-INFO-003</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -795,19 +795,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ISTG-FW-CONF-002</t>
+          <t>ISTG-FW-INFO-004</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -817,19 +817,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Insecure Binary Compilation Options</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ISTG-FW-SCRT-001</t>
+          <t>ISTG-FW-CONF-001</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -839,19 +839,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Secrets Stored in Public Storage</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ISTG-FW-SCRT-002</t>
+          <t>ISTG-FW-CONF-002</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -861,19 +861,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Unencrypted Storage of Secrets</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ISTG-FW-SCRT-003</t>
+          <t>ISTG-FW-SCRT-001</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -888,14 +888,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Usage of Hardcoded Secrets</t>
+          <t>Secrets Stored in Public Storage</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ISTG-FW-CRYPT-001</t>
+          <t>ISTG-FW-SCRT-002</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -905,63 +905,63 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Unencrypted Storage of Secrets</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ISTG-FW[INST]-AUTHZ-001</t>
+          <t>ISTG-FW-SCRT-003</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Installed Firmware</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Firmware</t>
+          <t>Usage of Hardcoded Secrets</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ISTG-FW[INST]-AUTHZ-002</t>
+          <t>ISTG-FW-CRYPT-001</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Installed Firmware</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ISTG-FW[INST]-INFO-001</t>
+          <t>ISTG-FW[INST]-AUTHZ-001</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -971,19 +971,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Unauthorized Access to the Firmware</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ISTG-FW[INST]-CRYPT-001</t>
+          <t>ISTG-FW[INST]-AUTHZ-002</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -993,46 +993,46 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Insufficient Verification of the Bootloader Signature</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ISTG-FW[UPDT]-AUTHZ-001</t>
+          <t>ISTG-FW[INST]-INFO-001</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Firmware Update Mechanism</t>
+          <t>Installed Firmware</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Unauthorized Firmware Update</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ISTG-FW[UPDT]-CRYPT-001</t>
+          <t>ISTG-FW[INST]-CRYPT-001</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Firmware Update Mechanism</t>
+          <t>Installed Firmware</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1042,14 +1042,14 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Insufficient Firmware Update Signature</t>
+          <t>Insufficient Verification of the Bootloader Signature</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ISTG-FW[UPDT]-CRYPT-002</t>
+          <t>ISTG-FW[UPDT]-AUTHZ-001</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1059,19 +1059,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Insufficient Firmware Update Encryption</t>
+          <t>Unauthorized Firmware Update</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ISTG-FW[UPDT]-CRYPT-003</t>
+          <t>ISTG-FW[UPDT]-CRYPT-001</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1086,14 +1086,14 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Insecure Transmission of the Firmware Update</t>
+          <t>Insufficient Firmware Update Signature</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ISTG-FW[UPDT]-CRYPT-004</t>
+          <t>ISTG-FW[UPDT]-CRYPT-002</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1108,14 +1108,14 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Insufficient Verification of the Firmware Update Signature</t>
+          <t>Insufficient Firmware Update Encryption</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ISTG-FW[UPDT]-LOGIC-001</t>
+          <t>ISTG-FW[UPDT]-CRYPT-003</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1125,63 +1125,63 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Insufficient Rollback Protection</t>
+          <t>Insecure Transmission of the Firmware Update</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ISTG-DES-AUTHZ-001</t>
+          <t>ISTG-FW[UPDT]-CRYPT-004</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Data Exchange Services</t>
+          <t>Firmware Update Mechanism</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Data Exchange Service</t>
+          <t>Insufficient Verification of the Firmware Update Signature</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ISTG-DES-AUTHZ-002</t>
+          <t>ISTG-FW[UPDT]-LOGIC-001</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Data Exchange Services</t>
+          <t>Firmware Update Mechanism</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Insufficient Rollback Protection</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ISTG-DES-INFO-001</t>
+          <t>ISTG-DES-AUTHZ-001</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1191,19 +1191,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Unauthorized Access to the Data Exchange Service</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ISTG-DES-INFO-002</t>
+          <t>ISTG-DES-AUTHZ-002</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1213,19 +1213,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ISTG-DES-INFO-003</t>
+          <t>ISTG-DES-INFO-001</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1240,14 +1240,14 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ISTG-DES-CONF-001</t>
+          <t>ISTG-DES-INFO-002</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1257,19 +1257,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ISTG-DES-CONF-002</t>
+          <t>ISTG-DES-INFO-003</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1279,19 +1279,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ISTG-DES-SCRT-001</t>
+          <t>ISTG-DES-CONF-001</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1301,19 +1301,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ISTG-DES-CRYPT-001</t>
+          <t>ISTG-DES-CONF-002</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1323,19 +1323,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ISTG-DES-LOGIC-001</t>
+          <t>ISTG-DES-SCRT-001</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1345,19 +1345,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ISTG-DES-INPV-001</t>
+          <t>ISTG-DES-CRYPT-001</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1367,19 +1367,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ISTG-DES-INPV-002</t>
+          <t>ISTG-DES-LOGIC-001</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1389,63 +1389,63 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ISTG-INT-AUTHZ-001</t>
+          <t>ISTG-DES-INPV-001</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Internal Interfaces</t>
+          <t>Data Exchange Services</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ISTG-INT-AUTHZ-002</t>
+          <t>ISTG-DES-INPV-002</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Internal Interfaces</t>
+          <t>Data Exchange Services</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ISTG-INT-INFO-001</t>
+          <t>ISTG-INT-AUTHZ-001</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1455,19 +1455,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ISTG-INT-INFO-002</t>
+          <t>ISTG-INT-AUTHZ-002</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1477,19 +1477,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ISTG-INT-INFO-003</t>
+          <t>ISTG-INT-INFO-001</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1504,14 +1504,14 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ISTG-INT-CONF-001</t>
+          <t>ISTG-INT-INFO-002</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1521,19 +1521,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ISTG-INT-CONF-002</t>
+          <t>ISTG-INT-INFO-003</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1543,19 +1543,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ISTG-INT-SCRT-001</t>
+          <t>ISTG-INT-CONF-001</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1565,19 +1565,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ISTG-INT-CRYPT-001</t>
+          <t>ISTG-INT-CONF-002</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1587,19 +1587,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ISTG-INT-LOGIC-001</t>
+          <t>ISTG-INT-SCRT-001</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1609,19 +1609,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ISTG-INT-INPV-001</t>
+          <t>ISTG-INT-CRYPT-001</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1631,19 +1631,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ISTG-INT-INPV-002</t>
+          <t>ISTG-INT-LOGIC-001</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1653,19 +1653,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ISTG-INT[JTAG]-AUTHZ-001</t>
+          <t>ISTG-INT-INPV-001</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1675,19 +1675,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Unauthorized Debug Access in Production State</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ISTG-INT[JTAG]-AUTHZ-002</t>
+          <t>ISTG-INT-INPV-002</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1697,46 +1697,46 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Early-Boot Debug-State Exposure</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ISTG-INT[JTAG]-INFO-001</t>
+          <t>ISTG-INT[I2C]-AUTHZ-001</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Internal Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Interface Presence, Physical Accessibility, and Transport Identification</t>
+          <t>Bus Interaction with Unauthorized Devices</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ISTG-INT[JTAG]-INFO-002</t>
+          <t>ISTG-INT[I2C]-INFO-001</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Internal Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1746,129 +1746,129 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Accessible Asset Boundary Review</t>
+          <t>Slave Enumeration</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ISTG-INT[JTAG]-CONF-001</t>
+          <t>ISTG-INT[I2C]-INFO-002</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Internal Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Lifecycle and Security-Configuration Review</t>
+          <t>Communication Sniffing</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ISTG-PHY-AUTHZ-001</t>
+          <t>ISTG-INT[I2C]-INFO-003</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>EEPROM/Memory Extraction</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ISTG-PHY-AUTHZ-002</t>
+          <t>ISTG-INT[I2C]-INPV-001</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Inter-Integrated Circuit</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Insufficient Handling of Invalid Data</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-001</t>
+          <t>ISTG-INT[UART]-AUTHZ-001</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Universal Asynchronous Receiver-Transmitter</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Unauthenticated Access to Serial Console</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-002</t>
+          <t>ISTG-INT[UART]-AUTHZ-002</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Universal Asynchronous Receiver-Transmitter</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Bootloader Interrupt via Serial Console</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INFO-003</t>
+          <t>ISTG-INT[UART]-INFO-001</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Universal Asynchronous Receiver-Transmitter</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1878,58 +1878,58 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>UART Interface and Baud Rate Identification</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CONF-001</t>
+          <t>ISTG-INT[UART]-INFO-002</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Universal Asynchronous Receiver-Transmitter</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Disclosure of Sensitive Data in Serial Output</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CONF-002</t>
+          <t>ISTG-INT[UART]-INPV-001</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Physical Interfaces</t>
+          <t>Universal Asynchronous Receiver-Transmitter</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Command Injection via Serial Interface</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ISTG-PHY-SCRT-001</t>
+          <t>ISTG-PHY-AUTHZ-001</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1939,19 +1939,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ISTG-PHY-CRYPT-001</t>
+          <t>ISTG-PHY-AUTHZ-002</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1961,19 +1961,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ISTG-PHY-LOGIC-001</t>
+          <t>ISTG-PHY-INFO-001</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1983,19 +1983,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INPV-001</t>
+          <t>ISTG-PHY-INFO-002</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2005,19 +2005,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ISTG-PHY-INPV-002</t>
+          <t>ISTG-PHY-INFO-003</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2027,173 +2027,173 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-AUTHZ-001</t>
+          <t>ISTG-PHY-CONF-001</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-AUTHZ-002</t>
+          <t>ISTG-PHY-CONF-002</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-001</t>
+          <t>ISTG-PHY-SCRT-001</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-002</t>
+          <t>ISTG-PHY-CRYPT-001</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INFO-003</t>
+          <t>ISTG-PHY-LOGIC-001</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CONF-001</t>
+          <t>ISTG-PHY-INPV-001</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CONF-002</t>
+          <t>ISTG-PHY-INPV-002</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Wireless Interfaces</t>
+          <t>Physical Interfaces</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-SCRT-001</t>
+          <t>ISTG-WRLS-AUTHZ-001</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2203,19 +2203,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-CRYPT-001</t>
+          <t>ISTG-WRLS-AUTHZ-002</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2225,19 +2225,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-LOGIC-001</t>
+          <t>ISTG-WRLS-INFO-001</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2247,19 +2247,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INPV-001</t>
+          <t>ISTG-WRLS-INFO-002</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ISTG-WRLS-INPV-002</t>
+          <t>ISTG-WRLS-INFO-003</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2291,173 +2291,173 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Code or Command Injection</t>
+          <t>Disclosure of User Data</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ISTG-UI-AUTHZ-001</t>
+          <t>ISTG-WRLS-CONF-001</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Unauthorized Access to the Interface</t>
+          <t>Usage of Outdated Software</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ISTG-UI-AUTHZ-002</t>
+          <t>ISTG-WRLS-CONF-002</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Authorization</t>
+          <t>Configuration and Patch Management</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Privilege Escalation</t>
+          <t>Presence of Unnecessary Software and Functionalities</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-001</t>
+          <t>ISTG-WRLS-SCRT-001</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Secrets</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Disclosure of Implementation Details</t>
+          <t>Access to Confidential Data</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-002</t>
+          <t>ISTG-WRLS-CRYPT-001</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Cryptography</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Disclosure of Ecosystem Details</t>
+          <t>Usage of Weak Cryptographic Algorithms</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ISTG-UI-INFO-003</t>
+          <t>ISTG-WRLS-LOGIC-001</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Information Gathering</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Disclosure of User Data</t>
+          <t>Circumvention of the Intended Business Logic</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ISTG-UI-CONF-001</t>
+          <t>ISTG-WRLS-INPV-001</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Usage of Outdated Software</t>
+          <t>Insufficient Input Validation</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ISTG-UI-CONF-002</t>
+          <t>ISTG-WRLS-INPV-002</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>User Interfaces</t>
+          <t>Wireless Interfaces</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Configuration and Patch Management</t>
+          <t>Input Validation</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Presence of Unnecessary Software and Functionalities</t>
+          <t>Code or Command Injection</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ISTG-UI-SCRT-001</t>
+          <t>ISTG-UI-AUTHZ-001</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2467,19 +2467,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Secrets</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Access to Confidential Data</t>
+          <t>Unauthorized Access to the Interface</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ISTG-UI-CRYPT-001</t>
+          <t>ISTG-UI-AUTHZ-002</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2489,19 +2489,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Usage of Weak Cryptographic Algorithms</t>
+          <t>Privilege Escalation</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ISTG-UI-LOGIC-001</t>
+          <t>ISTG-UI-INFO-001</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2511,19 +2511,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Business Logic</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Circumvention of the Intended Business Logic</t>
+          <t>Disclosure of Implementation Details</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ISTG-UI-INPV-001</t>
+          <t>ISTG-UI-INFO-002</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2533,32 +2533,186 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Input Validation</t>
+          <t>Information Gathering</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Insufficient Input Validation</t>
+          <t>Disclosure of Ecosystem Details</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
+          <t>ISTG-UI-INFO-003</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Information Gathering</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Disclosure of User Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ISTG-UI-CONF-001</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Configuration and Patch Management</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Usage of Outdated Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ISTG-UI-CONF-002</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Configuration and Patch Management</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Presence of Unnecessary Software and Functionalities</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ISTG-UI-SCRT-001</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Secrets</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Access to Confidential Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ISTG-UI-CRYPT-001</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Cryptography</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Usage of Weak Cryptographic Algorithms</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>ISTG-UI-LOGIC-001</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Business Logic</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Circumvention of the Intended Business Logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>ISTG-UI-INPV-001</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>User Interfaces</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Input Validation</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Insufficient Input Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>ISTG-UI-INPV-002</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>User Interfaces</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>Input Validation</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>Code or Command Injection</t>
         </is>

</xml_diff>